<commit_message>
fixed some xpaths and handle stale element exception
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testdata.xlsx
+++ b/src/test/resources/testData/testdata.xlsx
@@ -8,12 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\JAVA LEARNING\selenium\com.OrangeHRM\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB3A0B2-D26C-45BB-8321-D27D75D1A61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D0BE34-F8F2-4EEF-93B6-049610C8AF68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{128B943B-2108-4BC1-96AC-EC69D353BBE2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{128B943B-2108-4BC1-96AC-EC69D353BBE2}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
+    <sheet name="jobTitles" sheetId="2" r:id="rId2"/>
+    <sheet name="jobCategory" sheetId="3" r:id="rId3"/>
+    <sheet name="subUnits" sheetId="4" r:id="rId4"/>
+    <sheet name="employmentStatus" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>UserName</t>
   </si>
@@ -46,6 +50,183 @@
   </si>
   <si>
     <t>Valid</t>
+  </si>
+  <si>
+    <t>HR Manager</t>
+  </si>
+  <si>
+    <t>Software Engineer</t>
+  </si>
+  <si>
+    <t>QA Engineer</t>
+  </si>
+  <si>
+    <t>IT Manager</t>
+  </si>
+  <si>
+    <t>Sales Representative</t>
+  </si>
+  <si>
+    <t>Support Specialist</t>
+  </si>
+  <si>
+    <t>Account Assistant</t>
+  </si>
+  <si>
+    <t>Automaton Tester</t>
+  </si>
+  <si>
+    <t>Chief Executive Officer</t>
+  </si>
+  <si>
+    <t>Chief Financial Officer</t>
+  </si>
+  <si>
+    <t>Chief Technical Officer</t>
+  </si>
+  <si>
+    <t>Content Specialist</t>
+  </si>
+  <si>
+    <t>Customer Success Manager</t>
+  </si>
+  <si>
+    <t>Database Administrator</t>
+  </si>
+  <si>
+    <t>Finance Manager</t>
+  </si>
+  <si>
+    <t>Financial Analyst</t>
+  </si>
+  <si>
+    <t>Head of Support</t>
+  </si>
+  <si>
+    <t>HR Associate</t>
+  </si>
+  <si>
+    <t>Network Administrator</t>
+  </si>
+  <si>
+    <t>Payroll Administrator</t>
+  </si>
+  <si>
+    <t>Pre-Sales Coordinator</t>
+  </si>
+  <si>
+    <t>QA Lead</t>
+  </si>
+  <si>
+    <t>qwer</t>
+  </si>
+  <si>
+    <t>rsjsrii</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>Social Media Marketer</t>
+  </si>
+  <si>
+    <t>Software Architect</t>
+  </si>
+  <si>
+    <t>TestJob</t>
+  </si>
+  <si>
+    <t>VP - Client Services</t>
+  </si>
+  <si>
+    <t>VP - Sales &amp; Marketing</t>
+  </si>
+  <si>
+    <t>Craft Workers</t>
+  </si>
+  <si>
+    <t>Laborers and Helpers</t>
+  </si>
+  <si>
+    <t>Office and Clerical Workers</t>
+  </si>
+  <si>
+    <t>Officials and Managers</t>
+  </si>
+  <si>
+    <t>Operatives</t>
+  </si>
+  <si>
+    <t>Professionals</t>
+  </si>
+  <si>
+    <t>Sales Workers</t>
+  </si>
+  <si>
+    <t>Service Workers</t>
+  </si>
+  <si>
+    <t>Technicians</t>
+  </si>
+  <si>
+    <t>Administration</t>
+  </si>
+  <si>
+    <t>Engineering</t>
+  </si>
+  <si>
+    <t>Development</t>
+  </si>
+  <si>
+    <t>Quality Assurance</t>
+  </si>
+  <si>
+    <t>TechOps</t>
+  </si>
+  <si>
+    <t>Sales &amp; Marketing</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Client Services</t>
+  </si>
+  <si>
+    <t>Technical Support</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>hola</t>
+  </si>
+  <si>
+    <t>juan perez</t>
+  </si>
+  <si>
+    <t>Freelance</t>
+  </si>
+  <si>
+    <t>Full-Time Contract</t>
+  </si>
+  <si>
+    <t>Full-Time Permanent</t>
+  </si>
+  <si>
+    <t>Full-Time Probation</t>
+  </si>
+  <si>
+    <t>Part-Time Contract</t>
+  </si>
+  <si>
+    <t>Part-Time Internship</t>
   </si>
 </sst>
 </file>
@@ -96,9 +277,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,4 +636,351 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{135D514D-2763-4AAC-8228-E75300FDF9CA}">
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65B6C939-8E74-4223-AB28-C58BE3D56B7A}">
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0C3E025-67BA-4628-B388-992920C98BF4}">
+  <dimension ref="A1:A14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59DF2CD1-3910-4758-B94A-AC3D8FB3D57F}">
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>